<commit_message>
Add Excel template generation script and update template file handling
- Introduce `generate:templates` script in package.json for generating Excel templates.
- Refactor Excel template file handling in frontend to dynamically map template topics to file paths.
- Update multiple Excel files in the frontend/data directory to reflect new template structure.
</commit_message>
<xml_diff>
--- a/frontend/data/Hậu cần.xlsx
+++ b/frontend/data/Hậu cần.xlsx
@@ -1,118 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B6E4FB6-01FE-4F48-A474-36A6421A93CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
   <sheets>
-    <sheet name="Tu luan 2 cot" sheetId="1" r:id="rId1"/>
+    <sheet name="Hậu cần" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>Câu hỏi</t>
-  </si>
-  <si>
-    <t>Đáp án mẫu</t>
-  </si>
-  <si>
-    <t>1. Gạo tẻ 
-Toàn Sư đoàn dự trữ 05 ngày. Trung đoàn dự trữ 04 ngày, trong đó đầu mối các bếp ăn dự trữ 03 ngày, kho hậu cần trung đoàn dự trữ 01 ngày.
-Định lượng dự trữ: 700g/người/ngày
-2. Củi
-Toàn trung đoàn dự trữ 05 ngày tại đầu mối các đơn vị.
- Định lượng dự trữ: 700g/ng/ngày.</t>
-  </si>
-  <si>
-    <r>
-      <t>Đ/c cho biết lượng dự trữ gạo tẻ, c</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>ủi cho nhiệm vụ đột xuất trong công tác hậu cần SSCĐ?</t>
-    </r>
-  </si>
-  <si>
-    <t>Đ/c cho biết các loại thực phẩm và tiền ăn dự trữ cho nhiệm vụ đột xuất trong công tác hậu cần SSCĐ?</t>
-  </si>
-  <si>
-    <t>a) Thực phẩm (dự trữ 3 ngày)
-- Cá hộp: 1 hộp/ngày/6 người;	
-- Nước mắm: 30 ml/người/ngày;
-- Củ quả: 200 gam/người/ngày;	
-- Dầu ăn: 25ml/người/ngày.
-- Mì chính: 02 gam/người/ngày;
-Các loại thực phẩm dự trữ trên giá, trong kho thực phẩm tại nhà bếp, khi báo động phân theo đầu mối các trung đội, đại đội mang theo. Riêng củ quả khi báo động chỉ mang theo 60g/người/ngày.
-b) Tiền ăn
-Khi báo động kiểm tra, ngoài LTTP đơn vị còn phải mang theo lượng tiền ăn nhất định. Qua tính toán định lượng, giá cả hiện nay, số tiền được quy đổi từ LTTP, chất đốt khoảng 25.000đ/người/ngày. Số tiền mặt phải mang theo khi báo động thực hiện nhiệm vụ là: 65.000 - 25.000 = 40.000đ/người/ngày. Quân số khi báo động kiểm tra bao nhiêu thì nhân với 3 ngày tương ứng.</t>
-  </si>
-  <si>
-    <t>Đ/c cho biết tiêu chuẩn điện nước?</t>
-  </si>
-  <si>
-    <t>Tiêu chuẩn điện sinh hoạt: HSQ-CS: 11kw/người/tháng; Cấp úy: 28kw/người/tháng; Cấp thiếu, trung tá: 38kw/người/tháng.
-Tiêu chuẩn nước sinh hoạt: 140 lít/người/ngày.</t>
-  </si>
-  <si>
-    <t>Đ/c cho biết tiêu chuẩn bảo đảm ăn trong Công tác hậu cần thường xuyên?</t>
-  </si>
-  <si>
-    <t>Thực hiện theo Thông tư 168/TT-BQP ngày 18/12/2021 quy định tiêu chuẩn, định lượng, mức ăn cơ bản của Bộ binh = 65.000 đ/người/ngày; 12 ngày ăn thêm lễ tết.</t>
-  </si>
-  <si>
-    <t>Đ/c cho biết Tiêu chuẩn doanh cụ sinh hoạt?</t>
-  </si>
-  <si>
-    <t>HSQ-CS: 06 người/01 bộ (02 chậu to, 02 chậu nhỏ, 02 xô).
-SQ-QNCN: 04 người/01 bộ.</t>
-  </si>
-  <si>
-    <t>Đ/c cho biết Hệ số phụ cấp của Binh nhì?</t>
-  </si>
-  <si>
-    <t>0.4 lần lương cơ bản</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -135,26 +64,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -479,73 +396,48 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="55.81640625" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D3"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Câu hỏi</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Phương án</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Đáp án đúng</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Câu trả lời</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="121.2" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>(Nhập nội dung câu hỏi trắc nghiệm)</v>
+      </c>
+      <c r="B2" t="str" xml:space="preserve">
+        <v xml:space="preserve">A. Đáp án A_x000d_
+B. Đáp án B_x000d_
+C. Đáp án C_x000d_
+D. Đáp án D</v>
+      </c>
+      <c r="C2" t="str">
+        <v>A. Đáp án A</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="255" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="15" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>13</v>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>(Nhập nội dung câu hỏi tự luận)</v>
+      </c>
+      <c r="D3" t="str">
+        <v>(Nhập đáp án mẫu — Enter để xuống dòng)</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:B1" numberStoredAsText="1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>